<commit_message>
docs(seguimiento): P23-08 en progreso; borrador de las secciones corregidas sobre el alcance de la IA
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -7767,7 +7767,7 @@
       </c>
       <c r="F116" s="51" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="G116" s="51" t="inlineStr">
@@ -7777,12 +7777,12 @@
       </c>
       <c r="H116" s="51" t="inlineStr">
         <is>
-          <t>Plan 23, sección 6.</t>
+          <t>Plan 23, sección 6. Borrador de los textos de reemplazo: Documentacion/StockPilot_Secciones_corregidas_sobre_la_IA.docx (mismo formato que «Plan de Negocio — Secciones corregidas v2»).</t>
         </is>
       </c>
       <c r="I116" s="51" t="inlineStr">
         <is>
-          <t>Consultar al docente antes de cambiar título y objetivos. Verificar las citas contra los .docx originales.</t>
+          <t>Falta que Luis aplique los reemplazos en los documentos originales y consulte al docente antes de cambiar título y objetivos. Verificar los pasajes en Word (se ubicaron en textos extraídos). Seis verificaciones pendientes en la última página del borrador.</t>
         </is>
       </c>
       <c r="J116" s="51" t="inlineStr">
@@ -7925,7 +7925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="32" min="1" max="1"/>
@@ -8225,29 +8225,59 @@
       <c r="A13" s="53" t="n">
         <v>46301</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>P19-06, P11-02, P23-01 a P23-09</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="32" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="32" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="32" t="inlineStr">
         <is>
           <t>Decisiones del 6-oct: la IA va disponible pero opcional (oculta en el modo básico); se invertirá en corregir el evaluador y medir, contexto real al ajuste y lectura de facturas (plan 23); privacidad primero. Modo básico A, B y C implementado en la rama feat/modo-basico-web (subida). Arreglo de privacidad de Cartera (afddd1d) terminado. Rama del backend y 4 ramas de la app subidas; main sin tocar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" s="33">
+      <c r="A14" s="53" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>P23-08</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>En progreso</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Borrador de las secciones corregidas sobre el alcance de la IA, con el formato del documento «Secciones corregidas v2»: Documentacion/StockPilot_Secciones_corregidas_sobre_la_IA.docx (21 recuadros de instrucción, 4 tablas). Pendiente de que Luis lo aplique.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(seguimiento): P23-08 apunta a la Revisión v2 consolidada del Documento 5
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -7777,12 +7777,12 @@
       </c>
       <c r="H116" s="51" t="inlineStr">
         <is>
-          <t>Plan 23, sección 6. Borrador de los textos de reemplazo: Documentacion/StockPilot_Secciones_corregidas_sobre_la_IA.docx (mismo formato que «Plan de Negocio — Secciones corregidas v2»).</t>
+          <t>Plan 23, sección 6. Documento único para actualizar el Documento 5 del Drive: Documentacion/Revision_Documento_Practica_5_v2.docx (secciones A a G de la revisión del 26-sep, actualizadas, más H a K nuevas). Reemplaza al borrador «Secciones corregidas sobre la IA».</t>
         </is>
       </c>
       <c r="I116" s="51" t="inlineStr">
         <is>
-          <t>Falta que Luis aplique los reemplazos en los documentos originales y consulte al docente antes de cambiar título y objetivos. Verificar los pasajes en Word (se ubicaron en textos extraídos). Seis verificaciones pendientes en la última página del borrador.</t>
+          <t>Falta que Luis aplique los textos en el Documento 5 y en el Plan de Negocio e Intervención, y que consulte al docente antes de cambiar título y objetivos. Verificar los pasajes en Word/Drive. Nueve verificaciones pendientes en la sección K de la revisión v2.</t>
         </is>
       </c>
       <c r="J116" s="51" t="inlineStr">
@@ -7925,7 +7925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="32" min="1" max="1"/>
@@ -8255,29 +8255,59 @@
       <c r="A14" s="53" t="n">
         <v>46301</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
         <is>
           <t>P23-08</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="32" t="inlineStr">
         <is>
           <t>No iniciado</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="32" t="inlineStr">
         <is>
           <t>En progreso</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="32" t="inlineStr">
         <is>
           <t>Agente (Claude Code)</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="32" t="inlineStr">
         <is>
           <t>Borrador de las secciones corregidas sobre el alcance de la IA, con el formato del documento «Secciones corregidas v2»: Documentacion/StockPilot_Secciones_corregidas_sobre_la_IA.docx (21 recuadros de instrucción, 4 tablas). Pendiente de que Luis lo aplique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" s="33">
+      <c r="A15" s="53" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>P23-08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>En progreso</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>En progreso</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Se consolidó todo en Documentacion/Revision_Documento_Practica_5_v2.docx (24 páginas en Word, 10 tablas): revisión del 26-sep actualizada al 6-oct (pruebas 287 + 407, 28,2 KLOC, escáner, rol «Colaborador»), reglas de alertas, textos de la IA, novedades y correcciones a Plan de Negocio, Intervención y Herramientas. Se retira el borrador anterior «Secciones corregidas sobre la IA».</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(planes): R1 hecha en rama, resultados, hallazgos P21-17 a P21-22 y seguimiento actualizado
Plan 21: estado (8-oct), seccion «R1 — Resultados» (commits, estructura final
de services/ia, criterio de salida verificado, lo que no se movio, leccion del
primer intento, mutaciones, lint, evidencia y cobertura combinada 73,5 %) y 6
hallazgos nuevos. Tabla de tramos y decision 2 al dia.

Planes 20, 22, 23, plan_sprints (6.3) y hoja_de_ruta: rutas y referencias a
aiController / utils al estado actual de la rama (las del plan 20 como nota
historica).

seguimiento_planes.xlsx: P21-02 (R1) pasa a «Por verificar» (hecha en rama, sin
mezclar, igual que se trato R0 el 28-sep); notas en P21-03, P21-05 y P21-15;
filas P21-17 a P21-22; entrada en la Bitacora. Verificado abriendo una copia en
Excel: el resumen recalcula (119 pendientes).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -1697,7 +1697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="32" min="1" max="1"/>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="F75" s="51" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>Por verificar</t>
         </is>
       </c>
       <c r="G75" s="51" t="inlineStr">
@@ -5538,17 +5538,21 @@
       </c>
       <c r="H75" s="51" t="inlineStr">
         <is>
-          <t>Plan 21, sección 4.</t>
+          <t>Rama refactor/R1-servicios-ia, 6 commits (9ac27a4, 72b35c8, f01bbd0, 9306750, 458118e, b899d45). aiController 901 → 152 líneas; cliente único de OpenAI; services/ia/ con 14 módulos. 365 unitarias + 431 de integración en verde; cobertura combinada 73,5 %. Plan 21, «R1 — Resultados».</t>
         </is>
       </c>
       <c r="I75" s="51" t="inlineStr">
         <is>
-          <t>Después del piloto, salvo que la fecha del Sprint 6.3 lo exija antes.</t>
-        </is>
-      </c>
-      <c r="J75" s="51" t="n"/>
+          <t>Falta que Luis la apruebe y la mezcle a main. Se despliega después del piloto (congelamiento).</t>
+        </is>
+      </c>
+      <c r="J75" s="51" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
       <c r="K75" s="53" t="n">
-        <v>46292</v>
+        <v>46303</v>
       </c>
       <c r="L75" s="54">
         <f>IF(K75="","",TODAY()-K75)</f>
@@ -5596,10 +5600,14 @@
           <t>Plan 21, sección 4.</t>
         </is>
       </c>
-      <c r="I76" s="51" t="n"/>
+      <c r="I76" s="51" t="inlineStr">
+        <is>
+          <t>Antes de R2, caracterizar también las ramas de error de cada endpoint (lección de R1). suppliersController es hoy el controlador más grande (632 líneas) y conserva el prompt de generateSmartOrder.</t>
+        </is>
+      </c>
       <c r="J76" s="51" t="n"/>
       <c r="K76" s="53" t="n">
-        <v>46292</v>
+        <v>46303</v>
       </c>
       <c r="L76" s="54">
         <f>IF(K76="","",TODAY()-K76)</f>
@@ -5702,10 +5710,14 @@
           <t>Plan 21, sección 4.</t>
         </is>
       </c>
-      <c r="I78" s="51" t="n"/>
+      <c r="I78" s="51" t="inlineStr">
+        <is>
+          <t>Al 8-oct quedan 164 console.* en el backend (authController 24, schedulerService 15, saleController 12, productController 12, app.js 12…). R1 limpió aiController, services/ia, services/inventory y suppliersController. Incluir mover ai_audit.log de la raíz a logs/.</t>
+        </is>
+      </c>
       <c r="J78" s="51" t="n"/>
       <c r="K78" s="53" t="n">
-        <v>46292</v>
+        <v>46303</v>
       </c>
       <c r="L78" s="54">
         <f>IF(K78="","",TODAY()-K78)</f>
@@ -6250,12 +6262,12 @@
       </c>
       <c r="I88" s="51" t="inlineStr">
         <is>
-          <t>Recomendado: sí, antes de tener datos reales en producción.</t>
+          <t>Recomendado: sí, antes de tener datos reales en producción. Ratificado el 8-oct: cargar cualquier módulo que importe config/database.js dispara la auto-migración contra el DATABASE_URL del .env (ocurrió por accidente al comprobar un require; apuntaba a la base local).</t>
         </is>
       </c>
       <c r="J88" s="51" t="n"/>
       <c r="K88" s="53" t="n">
-        <v>46292</v>
+        <v>46303</v>
       </c>
       <c r="L88" s="54">
         <f>IF(K88="","",TODAY()-K88)</f>
@@ -7854,6 +7866,348 @@
       </c>
       <c r="L117" s="54">
         <f>IF(K117="","",TODAY()-K117)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118" ht="23.85" customHeight="1" s="33">
+      <c r="A118" s="51" t="inlineStr">
+        <is>
+          <t>P21-17</t>
+        </is>
+      </c>
+      <c r="B118" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C118" s="51" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="D118" s="51" t="inlineStr">
+        <is>
+          <t>generar_reporte.js escribía el reporte en Documentacion/ (carpeta que el commit a665b8c eliminó) y npm run test:evidence terminaba en verde sin generarlo</t>
+        </is>
+      </c>
+      <c r="E118" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F118" s="51" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G118" s="51" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H118" s="51" t="inlineStr">
+        <is>
+          <t>Corregido en b899d45 (rama refactor/R1-servicios-ia): ruta a docs/ y process.exitCode = 1 si falla. Reporte regenerado: 365 + 431 = 796 pruebas.</t>
+        </is>
+      </c>
+      <c r="I118" s="51" t="inlineStr">
+        <is>
+          <t>Mezclar la rama a main.</t>
+        </is>
+      </c>
+      <c r="J118" s="51" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K118" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L118" s="54">
+        <f>IF(K118="","",TODAY()-K118)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119" ht="23.85" customHeight="1" s="33">
+      <c r="A119" s="51" t="inlineStr">
+        <is>
+          <t>P21-18</t>
+        </is>
+      </c>
+      <c r="B119" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C119" s="51" t="inlineStr">
+        <is>
+          <t>Documentación</t>
+        </is>
+      </c>
+      <c r="D119" s="51" t="inlineStr">
+        <is>
+          <t>El CLAUDE.md del repo todavía cita Documentacion/Reporte_Pruebas_StockPilot.md; hoy el reporte está en docs/</t>
+        </is>
+      </c>
+      <c r="E119" s="51" t="inlineStr">
+        <is>
+          <t>Mantenimiento de docs</t>
+        </is>
+      </c>
+      <c r="F119" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G119" s="51" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H119" s="51" t="inlineStr">
+        <is>
+          <t>CLAUDE.md (sección «Antes de ejecutar comandos que escriben o regeneran archivos»).</t>
+        </is>
+      </c>
+      <c r="I119" s="51" t="inlineStr">
+        <is>
+          <t>Es un archivo de Luis: pendiente de que lo actualice.</t>
+        </is>
+      </c>
+      <c r="J119" s="51" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K119" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L119" s="54">
+        <f>IF(K119="","",TODAY()-K119)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120" ht="23.85" customHeight="1" s="33">
+      <c r="A120" s="51" t="inlineStr">
+        <is>
+          <t>P21-19</t>
+        </is>
+      </c>
+      <c r="B120" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C120" s="51" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="D120" s="51" t="inlineStr">
+        <is>
+          <t>coverage.include usa utils/**/*.js, que también cuenta 4 archivos de frontend/src/utils (arqueo, menu, pedir, security2FA; 126 sentencias al 100 %) en la cobertura del backend</t>
+        </is>
+      </c>
+      <c r="E120" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F120" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G120" s="51" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H120" s="51" t="inlineStr">
+        <is>
+          <t>vitest.config.js. Infla cerca de un punto la cobertura combinada (73,5 % reportado).</t>
+        </is>
+      </c>
+      <c r="I120" s="51" t="inlineStr">
+        <is>
+          <t>Acotar el patrón (p. ej. ./utils/**) o documentar que es intencional.</t>
+        </is>
+      </c>
+      <c r="J120" s="51" t="n"/>
+      <c r="K120" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L120" s="54">
+        <f>IF(K120="","",TODAY()-K120)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121" ht="23.85" customHeight="1" s="33">
+      <c r="A121" s="51" t="inlineStr">
+        <is>
+          <t>P21-20</t>
+        </is>
+      </c>
+      <c r="B121" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C121" s="51" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="D121" s="51" t="inlineStr">
+        <is>
+          <t>Los umbrales de cobertura unitaria (10/15/19/9) están muy por debajo de lo medido (18,3/25,5/35,1/17,1); el plan 21, sección 3, pide subirlos, nunca bajarlos</t>
+        </is>
+      </c>
+      <c r="E121" s="51" t="inlineStr">
+        <is>
+          <t>Decisión pendiente</t>
+        </is>
+      </c>
+      <c r="F121" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G121" s="51" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H121" s="51" t="inlineStr">
+        <is>
+          <t>vitest.config.js. Medido el 8-oct con npm run test:coverage:combinada.</t>
+        </is>
+      </c>
+      <c r="I121" s="51" t="inlineStr">
+        <is>
+          <t>Propuesta: 17/23/32/15 (un poco por debajo de lo medido). Es configuración de pruebas/CI: lo decide Luis.</t>
+        </is>
+      </c>
+      <c r="J121" s="51" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K121" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L121" s="54">
+        <f>IF(K121="","",TODAY()-K121)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122" ht="23.85" customHeight="1" s="33">
+      <c r="A122" s="51" t="inlineStr">
+        <is>
+          <t>P21-21</t>
+        </is>
+      </c>
+      <c r="B122" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C122" s="51" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="D122" s="51" t="inlineStr">
+        <is>
+          <t>Zonas con poca cobertura combinada: tenderoController 6 %, dashboardController 10 %, auditController 11 %, schedulerService 12 % (correos), storeController 30 %, reportController 40 %</t>
+        </is>
+      </c>
+      <c r="E122" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F122" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G122" s="51" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H122" s="51" t="inlineStr">
+        <is>
+          <t>Cobertura combinada del 8-oct (npm run test:coverage:combinada).</t>
+        </is>
+      </c>
+      <c r="I122" s="51" t="inlineStr">
+        <is>
+          <t>Caracterizarlas antes de R2 y R3. El planificador de correos es el de mayor riesgo.</t>
+        </is>
+      </c>
+      <c r="J122" s="51" t="n"/>
+      <c r="K122" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L122" s="54">
+        <f>IF(K122="","",TODAY()-K122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123" ht="23.85" customHeight="1" s="33">
+      <c r="A123" s="51" t="inlineStr">
+        <is>
+          <t>P21-22</t>
+        </is>
+      </c>
+      <c r="B123" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C123" s="51" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="D123" s="51" t="inlineStr">
+        <is>
+          <t>Las corridas de integración muestran MaxListenersExceededWarning (11 listeners en un Server, probablemente supertest con isolate:false)</t>
+        </is>
+      </c>
+      <c r="E123" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F123" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G123" s="51" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H123" s="51" t="inlineStr">
+        <is>
+          <t>Salida de npm run test:integration y de test:evidence (8-oct).</t>
+        </is>
+      </c>
+      <c r="I123" s="51" t="inlineStr">
+        <is>
+          <t>Inofensivo. Ya aparecía antes del cierre de R1; no se verificó si es anterior a R1.</t>
+        </is>
+      </c>
+      <c r="J123" s="51" t="n"/>
+      <c r="K123" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L123" s="54">
+        <f>IF(K123="","",TODAY()-K123)</f>
         <v/>
       </c>
     </row>
@@ -7925,7 +8279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="32" min="1" max="1"/>
@@ -8285,29 +8639,59 @@
       <c r="A15" s="53" t="n">
         <v>46301</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>P23-08</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="32" t="inlineStr">
         <is>
           <t>En progreso</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="32" t="inlineStr">
         <is>
           <t>En progreso</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="32" t="inlineStr">
         <is>
           <t>Agente (Claude Code)</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="32" t="inlineStr">
         <is>
           <t>Se consolidó todo en Documentacion/Revision_Documento_Practica_5_v2.docx (24 páginas en Word, 10 tablas): revisión del 26-sep actualizada al 6-oct (pruebas 287 + 407, 28,2 KLOC, escáner, rol «Colaborador»), reglas de alertas, textos de la IA, novedades y correcciones a Plan de Negocio, Intervención y Herramientas. Se retira el borrador anterior «Secciones corregidas sobre la IA».</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" s="33">
+      <c r="A16" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>P21-02, P21-17 a P21-22</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="inlineStr">
+        <is>
+          <t>No iniciado / —</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
+        <is>
+          <t>Por verificar / No iniciado</t>
+        </is>
+      </c>
+      <c r="E16" s="32" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="F16" s="32" t="inlineStr">
+        <is>
+          <t>R1 del plan 21 hecha en la rama refactor/R1-servicios-ia (6 commits, sin mezclar a main): aiController 901 → 152 líneas, cliente único de OpenAI, services/ia con 14 módulos. 365 unitarias + 431 de integración en verde (796 en el reporte); cobertura combinada 73,5 %. Hallazgos nuevos P21-17 a P21-22: reporte de pruebas en carpeta inexistente (corregido en la rama), ruta vieja en CLAUDE.md, umbrales de cobertura por subir (decisión de Luis), zonas con poca cobertura.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(planes): R1 aprobada y mezclada a main local; umbrales y CLAUDE.md resueltos; seguimiento al dia
Plan 21 (estado, resultados, hallazgos P21-18 y P21-20 resueltos, tabla de tramos),
plan 22 y plan_sprints con el estado real. seguimiento_planes.xlsx: P21-02, P21-17,
P21-18 y P21-20 pasan a Terminado, con entrada en la Bitacora. Se deja constancia de
que origin/main no se actualiza todavia (main local lleva 5 commits previos sin subir).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -5528,7 +5528,7 @@
       </c>
       <c r="F75" s="51" t="inlineStr">
         <is>
-          <t>Por verificar</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="G75" s="51" t="inlineStr">
@@ -5538,12 +5538,12 @@
       </c>
       <c r="H75" s="51" t="inlineStr">
         <is>
-          <t>Rama refactor/R1-servicios-ia, 6 commits (9ac27a4, 72b35c8, f01bbd0, 9306750, 458118e, b899d45). aiController 901 → 152 líneas; cliente único de OpenAI; services/ia/ con 14 módulos. 365 unitarias + 431 de integración en verde; cobertura combinada 73,5 %. Plan 21, «R1 — Resultados».</t>
+          <t>Rama refactor/R1-servicios-ia (subida) y merge --no-ff a main local el 8-oct. aiController 901 → 152 líneas; cliente único de OpenAI; services/ia/ con 14 módulos. 365 unitarias + 431 de integración en verde; cobertura combinada 73,5 %. Plan 21, «R1 — Resultados».</t>
         </is>
       </c>
       <c r="I75" s="51" t="inlineStr">
         <is>
-          <t>Falta que Luis la apruebe y la mezcle a main. Se despliega después del piloto (congelamiento).</t>
+          <t>Aprobada por Luis el 8-oct. origin/main NO se actualizó: main local tiene 5 commits previos sin subir (incluye el 2FA en CRUD) y subirlo podría desplegar durante el congelamiento. Se despliega después del piloto.</t>
         </is>
       </c>
       <c r="J75" s="51" t="inlineStr">
@@ -7897,7 +7897,7 @@
       </c>
       <c r="F118" s="51" t="inlineStr">
         <is>
-          <t>Por verificar</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="G118" s="51" t="inlineStr">
@@ -7912,7 +7912,7 @@
       </c>
       <c r="I118" s="51" t="inlineStr">
         <is>
-          <t>Mezclar la rama a main.</t>
+          <t>Mezclado a main local el 8-oct (commit b899d45). Falta subir main.</t>
         </is>
       </c>
       <c r="J118" s="51" t="inlineStr">
@@ -7956,7 +7956,7 @@
       </c>
       <c r="F119" s="51" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="G119" s="51" t="inlineStr">
@@ -7966,17 +7966,17 @@
       </c>
       <c r="H119" s="51" t="inlineStr">
         <is>
-          <t>CLAUDE.md (sección «Antes de ejecutar comandos que escriben o regeneran archivos»).</t>
+          <t>CLAUDE.md del repo; commit 6d7db26.</t>
         </is>
       </c>
       <c r="I119" s="51" t="inlineStr">
         <is>
-          <t>Es un archivo de Luis: pendiente de que lo actualice.</t>
+          <t>Corregido el 8-oct con la aprobación de Luis.</t>
         </is>
       </c>
       <c r="J119" s="51" t="inlineStr">
         <is>
-          <t>Luis</t>
+          <t>Agente (Claude Code)</t>
         </is>
       </c>
       <c r="K119" s="53" t="n">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="F121" s="51" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="G121" s="51" t="inlineStr">
@@ -8080,12 +8080,12 @@
       </c>
       <c r="H121" s="51" t="inlineStr">
         <is>
-          <t>vitest.config.js. Medido el 8-oct con npm run test:coverage:combinada.</t>
+          <t>vitest.config.js: umbrales unitarios 10/15/19/9 → 17/23/32/15 (commit 91d8537). Medido: 18,3/25,3/34,4/17,0; el control falla con código 1 si no se cumple.</t>
         </is>
       </c>
       <c r="I121" s="51" t="inlineStr">
         <is>
-          <t>Propuesta: 17/23/32/15 (un poco por debajo de lo medido). Es configuración de pruebas/CI: lo decide Luis.</t>
+          <t>Aprobado por Luis el 8-oct. Regla del plan 21, sección 3: los pisos solo suben.</t>
         </is>
       </c>
       <c r="J121" s="51" t="inlineStr">
@@ -8279,7 +8279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="32" min="1" max="1"/>
@@ -8692,6 +8692,36 @@
       <c r="F16" s="32" t="inlineStr">
         <is>
           <t>R1 del plan 21 hecha en la rama refactor/R1-servicios-ia (6 commits, sin mezclar a main): aiController 901 → 152 líneas, cliente único de OpenAI, services/ia con 14 módulos. 365 unitarias + 431 de integración en verde (796 en el reporte); cobertura combinada 73,5 %. Hallazgos nuevos P21-17 a P21-22: reporte de pruebas en carpeta inexistente (corregido en la rama), ruta vieja en CLAUDE.md, umbrales de cobertura por subir (decisión de Luis), zonas con poca cobertura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" s="33">
+      <c r="A17" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>P21-02, P21-17, P21-18, P21-20</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>Por verificar / No iniciado</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>Terminado</t>
+        </is>
+      </c>
+      <c r="E17" s="32" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>Luis aprueba R1 y manda mezclarla (8-oct): merge --no-ff a main local; la rama refactor/R1-servicios-ia se sube como evidencia. Aprueba también subir los umbrales de cobertura (17/23/32/15) y corregir la ruta vieja del CLAUDE.md. origin/main no se actualiza todavía: main local lleva 5 commits previos sin subir (incluido el 2FA en CRUD, ec4d48c) y no se sabe si subir main despliega durante el congelamiento. Regla de Luis: cada plan nuevo debe quedar subido, es la evidencia del desarrollo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(planes): main se sube a origin con R1; Luis autoriza el despliegue antes de la visita
Plan 21, plan 22 y plan_sprints: R1 queda mezclada y subida a main (ya no «main local»).
Se explica que main llevaba 5 commits previos sin subir (incluido el 2FA en CRUD) y que
el congelamiento del piloto rige desde su arranque. Seguimiento: notas de P21-02 y
P21-17 y entrada en la Bitacora.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -5538,12 +5538,12 @@
       </c>
       <c r="H75" s="51" t="inlineStr">
         <is>
-          <t>Rama refactor/R1-servicios-ia (subida) y merge --no-ff a main local el 8-oct. aiController 901 → 152 líneas; cliente único de OpenAI; services/ia/ con 14 módulos. 365 unitarias + 431 de integración en verde; cobertura combinada 73,5 %. Plan 21, «R1 — Resultados».</t>
+          <t>Merge --no-ff a main (f93958e) y main subido a origin el 8-oct, junto con la rama refactor/R1-servicios-ia. aiController 901 → 152 líneas; cliente único de OpenAI; services/ia/ con 14 módulos. 365 unitarias + 431 de integración en verde; cobertura combinada 73,5 %. Plan 21, «R1 — Resultados».</t>
         </is>
       </c>
       <c r="I75" s="51" t="inlineStr">
         <is>
-          <t>Aprobada por Luis el 8-oct. origin/main NO se actualizó: main local tiene 5 commits previos sin subir (incluye el 2FA en CRUD) y subirlo podría desplegar durante el congelamiento. Se despliega después del piloto.</t>
+          <t>Aprobada por Luis el 8-oct. Subir main publicó también 5 commits previos suyos (entre ellos el 2FA en CRUD, ec4d48c). Luis autorizó subir a producción: la visita a las tiendas aún no ocurre. Falta comprobar el despliegue en Render.</t>
         </is>
       </c>
       <c r="J75" s="51" t="inlineStr">
@@ -7912,7 +7912,7 @@
       </c>
       <c r="I118" s="51" t="inlineStr">
         <is>
-          <t>Mezclado a main local el 8-oct (commit b899d45). Falta subir main.</t>
+          <t>Subido a main el 8-oct (commit b899d45).</t>
         </is>
       </c>
       <c r="J118" s="51" t="inlineStr">
@@ -8279,7 +8279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="32" min="1" max="1"/>
@@ -8722,6 +8722,36 @@
       <c r="F17" s="32" t="inlineStr">
         <is>
           <t>Luis aprueba R1 y manda mezclarla (8-oct): merge --no-ff a main local; la rama refactor/R1-servicios-ia se sube como evidencia. Aprueba también subir los umbrales de cobertura (17/23/32/15) y corregir la ruta vieja del CLAUDE.md. origin/main no se actualiza todavía: main local lleva 5 commits previos sin subir (incluido el 2FA en CRUD, ec4d48c) y no se sabe si subir main despliega durante el congelamiento. Regla de Luis: cada plan nuevo debe quedar subido, es la evidencia del desarrollo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" s="33">
+      <c r="A18" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>P21-02, P21-17, P21-18, P21-20</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="inlineStr">
+        <is>
+          <t>Terminado</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <t>Terminado</t>
+        </is>
+      </c>
+      <c r="E18" s="32" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="F18" s="32" t="inlineStr">
+        <is>
+          <t>Luis autoriza subir a producción (8-oct): la visita a las tiendas aún no ocurre. Se sube main a origin con R1 y con 5 commits previos que estaban sin subir (incluido el 2FA en CRUD, ec4d48c). Se corrige lo anotado antes: ya no queda origin/main pendiente. El congelamiento del piloto rige desde su arranque.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(2fa): revision del commit ec4d48c, politica de 2FA y procedimiento de soporte; reporte de pruebas (372 + 449 = 821)
Plan 21: seccion «Revision del 2FA» con la decision de Luis (en el piloto se informa, no se
exige), lo que se hizo y los hallazgos P21-23 a P21-28 (codigos de recuperacion como
prerrequisito de encender la politica, secreto TOTP en texto plano, modal duplicado en el
perfil). Plan 22: tarea posterior al piloto. Protocolo_Produccion: seccion 5 con la variable
REQUIRE_ADMIN_2FA y el procedimiento para ayudar a un dueno que perdio el celular.
Seguimiento: filas P21-23 a P21-28 y Bitacora. Reporte regenerado con test:evidence.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -1697,7 +1697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="32" min="1" max="1"/>
@@ -8208,6 +8208,352 @@
       </c>
       <c r="L123" s="54">
         <f>IF(K123="","",TODAY()-K123)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124" ht="23.85" customHeight="1" s="33">
+      <c r="A124" s="51" t="inlineStr">
+        <is>
+          <t>P21-23</t>
+        </is>
+      </c>
+      <c r="B124" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C124" s="51" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D124" s="51" t="inlineStr">
+        <is>
+          <t>El 2FA «obligatorio» del commit ec4d48c solo existía en el navegador: la API aceptaba cualquier escritura de un Administrador sin 2FA</t>
+        </is>
+      </c>
+      <c r="E124" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F124" s="51" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G124" s="51" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H124" s="51" t="inlineStr">
+        <is>
+          <t>Rama feat/2fa-politica-servidor (commits de la política en el servidor y del frontend). middleware/twoFactor.js, 18 pruebas de integración. Verificado en el navegador contra stockpilot_test.</t>
+        </is>
+      </c>
+      <c r="I124" s="51" t="inlineStr">
+        <is>
+          <t>Apagada por defecto (REQUIRE_ADMIN_2FA); decisión de Luis del 8-oct: en el piloto se informa, no se exige. Falta mezclar a main.</t>
+        </is>
+      </c>
+      <c r="J124" s="51" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K124" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L124" s="54">
+        <f>IF(K124="","",TODAY()-K124)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125" ht="23.85" customHeight="1" s="33">
+      <c r="A125" s="51" t="inlineStr">
+        <is>
+          <t>P21-24</t>
+        </is>
+      </c>
+      <c r="B125" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C125" s="51" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D125" s="51" t="inlineStr">
+        <is>
+          <t>generate2FA sobrescribía el secreto de un 2FA ya activo sin pedir contraseña ni código (una sesión robada podía cambiar el segundo factor)</t>
+        </is>
+      </c>
+      <c r="E125" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F125" s="51" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G125" s="51" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H125" s="51" t="inlineStr">
+        <is>
+          <t>controllers/authController.js: 409 DOS_FACTORES_YA_ACTIVO. Cubierto en politica_dos_factores.test.js.</t>
+        </is>
+      </c>
+      <c r="I125" s="51" t="inlineStr">
+        <is>
+          <t>Falta mezclar a main.</t>
+        </is>
+      </c>
+      <c r="J125" s="51" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K125" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L125" s="54">
+        <f>IF(K125="","",TODAY()-K125)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126" ht="23.85" customHeight="1" s="33">
+      <c r="A126" s="51" t="inlineStr">
+        <is>
+          <t>P21-25</t>
+        </is>
+      </c>
+      <c r="B126" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C126" s="51" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D126" s="51" t="inlineStr">
+        <is>
+          <t>/api/2fa/generate y /api/2fa/disable no tenían limitador de intentos (disable pide la contraseña y se podía adivinar sin límite)</t>
+        </is>
+      </c>
+      <c r="E126" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F126" s="51" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G126" s="51" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H126" s="51" t="inlineStr">
+        <is>
+          <t>middleware/rateLimiter.js: twoFactorSetupLimiter (5 fallos / 15 min), aparte de twoFactorLimiter. Cubierto en politica_dos_factores.test.js.</t>
+        </is>
+      </c>
+      <c r="I126" s="51" t="inlineStr">
+        <is>
+          <t>Falta mezclar a main.</t>
+        </is>
+      </c>
+      <c r="J126" s="51" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K126" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L126" s="54">
+        <f>IF(K126="","",TODAY()-K126)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127" ht="23.85" customHeight="1" s="33">
+      <c r="A127" s="51" t="inlineStr">
+        <is>
+          <t>P21-26</t>
+        </is>
+      </c>
+      <c r="B127" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C127" s="51" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D127" s="51" t="inlineStr">
+        <is>
+          <t>Códigos de recuperación del 2FA: si un dueño pierde el celular queda fuera de su cuenta</t>
+        </is>
+      </c>
+      <c r="E127" s="51" t="inlineStr">
+        <is>
+          <t>Decisión pendiente</t>
+        </is>
+      </c>
+      <c r="F127" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G127" s="51" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H127" s="51" t="inlineStr">
+        <is>
+          <t>Plan 21, revisión del 2FA. Hoy solo existe el procedimiento manual de soporte (docs/Protocolo_Produccion.md, sección 5).</t>
+        </is>
+      </c>
+      <c r="I127" s="51" t="inlineStr">
+        <is>
+          <t>Prerrequisito de encender REQUIRE_ADMIN_2FA. Después del piloto.</t>
+        </is>
+      </c>
+      <c r="J127" s="51" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K127" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L127" s="54">
+        <f>IF(K127="","",TODAY()-K127)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128" ht="23.85" customHeight="1" s="33">
+      <c r="A128" s="51" t="inlineStr">
+        <is>
+          <t>P21-27</t>
+        </is>
+      </c>
+      <c r="B128" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C128" s="51" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D128" s="51" t="inlineStr">
+        <is>
+          <t>El secreto TOTP se guarda en texto plano en Usuarios.two_factor_secret y la ventana de tolerancia de otplib es la de por defecto</t>
+        </is>
+      </c>
+      <c r="E128" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F128" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G128" s="51" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H128" s="51" t="inlineStr">
+        <is>
+          <t>models/User.js (set2FASecret); controllers/authController.js (authenticator.check sin options).</t>
+        </is>
+      </c>
+      <c r="I128" s="51" t="inlineStr">
+        <is>
+          <t>Revisar el cifrado en reposo después del piloto.</t>
+        </is>
+      </c>
+      <c r="J128" s="51" t="n"/>
+      <c r="K128" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L128" s="54">
+        <f>IF(K128="","",TODAY()-K128)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129" ht="23.85" customHeight="1" s="33">
+      <c r="A129" s="51" t="inlineStr">
+        <is>
+          <t>P21-28</t>
+        </is>
+      </c>
+      <c r="B129" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C129" s="51" t="inlineStr">
+        <is>
+          <t>Refactorización</t>
+        </is>
+      </c>
+      <c r="D129" s="51" t="inlineStr">
+        <is>
+          <t>ProfilePage tiene su propio modal de activación del 2FA, copia del nuevo components/security/Activar2FAModal.jsx</t>
+        </is>
+      </c>
+      <c r="E129" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F129" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G129" s="51" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H129" s="51" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/ProfilePage.jsx (show2FAModal).</t>
+        </is>
+      </c>
+      <c r="I129" s="51" t="inlineStr">
+        <is>
+          <t>Unificar al tocar el perfil (R3).</t>
+        </is>
+      </c>
+      <c r="J129" s="51" t="n"/>
+      <c r="K129" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L129" s="54">
+        <f>IF(K129="","",TODAY()-K129)</f>
         <v/>
       </c>
     </row>
@@ -8279,7 +8625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="32" min="1" max="1"/>
@@ -8752,6 +9098,36 @@
       <c r="F18" s="32" t="inlineStr">
         <is>
           <t>Luis autoriza subir a producción (8-oct): la visita a las tiendas aún no ocurre. Se sube main a origin con R1 y con 5 commits previos que estaban sin subir (incluido el 2FA en CRUD, ec4d48c). Se corrige lo anotado antes: ya no queda origin/main pendiente. El congelamiento del piloto rige desde su arranque.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" s="33">
+      <c r="A19" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>P21-23 a P21-28</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>Por verificar / No iniciado</t>
+        </is>
+      </c>
+      <c r="E19" s="32" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>Revisión del 2FA del commit ec4d48c: era solo frontend. Luis decide que en el piloto el 2FA se informa pero no se exige, y aprueba mover el control al servidor como política apagada por defecto (REQUIRE_ADMIN_2FA). Rama feat/2fa-politica-servidor (política en el servidor, 409 en generate2FA, limitador, aviso en el frontend). Pendiente: mezclar a main, códigos de recuperación antes de encender la política.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(panel-interno): resultados de I1/I2, guia operativa de cuentas del equipo, definiciones pendientes y seguimiento
Plan 22: estado, tabla de fases y seccion «I1 e I2 — Resultados» (lo implementado, donde se aparta del diseno, las
3 definiciones PROPUESTAS que Luis debe confirmar, lo que queda de I4 y los hallazgos). Plan 21: P21-29 (carrera latente
del helper de pruebas). Protocolo_Produccion, seccion 6: como crear/desactivar cuentas del equipo, copia de seguridad
previa, marcar tiendas de prueba y seguridad del acceso. Seguimiento: P22-02, P22-03, P22-19 y P22-05 actualizadas;
filas P22-20 a P22-23 y P21-29; entrada en la Bitacora.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -1697,7 +1697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L129"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="32" min="1" max="1"/>
@@ -6412,7 +6412,7 @@
       </c>
       <c r="F91" s="51" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>Por verificar</t>
         </is>
       </c>
       <c r="G91" s="51" t="inlineStr">
@@ -6422,17 +6422,21 @@
       </c>
       <c r="H91" s="51" t="inlineStr">
         <is>
-          <t>Plan 22, secciones 3.1 y 3.2.</t>
+          <t>Rama feat/panel-interno-metricas (cc0cbc0, df92831). Esquema interno, cuentas del equipo por script (npm run equipo:crear), login con 2FA obligatorio, requireEquipo, bitácora. Probado: 34 de integración + script de punta a punta + navegador real.</t>
         </is>
       </c>
       <c r="I91" s="51" t="inlineStr">
         <is>
-          <t>Antes del arranque del piloto (plan 22, sección 5, C.2).</t>
-        </is>
-      </c>
-      <c r="J91" s="51" t="n"/>
+          <t>Falta mezclar a main y crear las cuentas en producción (docs/Protocolo_Produccion.md, sección 6).</t>
+        </is>
+      </c>
+      <c r="J91" s="51" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
       <c r="K91" s="53" t="n">
-        <v>46293</v>
+        <v>46303</v>
       </c>
       <c r="L91" s="54">
         <f>IF(K91="","",TODAY()-K91)</f>
@@ -6467,7 +6471,7 @@
       </c>
       <c r="F92" s="51" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>Por verificar</t>
         </is>
       </c>
       <c r="G92" s="51" t="inlineStr">
@@ -6477,17 +6481,21 @@
       </c>
       <c r="H92" s="51" t="inlineStr">
         <is>
-          <t>Plan 22, secciones 3.3 y 3.5.</t>
+          <t>Rama feat/panel-interno-metricas (cc0cbc0, df92831, eb0a7f2). Vistas v_tiendas_resumen/v_activacion/v_adopcion_semanal y pantallas Tiendas, Detalle, Embudo y Bitácora. 32 + 30 de integración. Funciona con una sola tienda.</t>
         </is>
       </c>
       <c r="I92" s="51" t="inlineStr">
         <is>
-          <t>Antes del arranque del piloto. Debe excluir las tiendas de prueba (P22-19).</t>
-        </is>
-      </c>
-      <c r="J92" s="51" t="n"/>
+          <t>Excluye las tiendas de prueba. Pendiente que Luis confirme 3 definiciones propuestas (P22-20 y P22-21).</t>
+        </is>
+      </c>
+      <c r="J92" s="51" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
       <c r="K92" s="53" t="n">
-        <v>46293</v>
+        <v>46303</v>
       </c>
       <c r="L92" s="54">
         <f>IF(K92="","",TODAY()-K92)</f>
@@ -6577,7 +6585,7 @@
       </c>
       <c r="F94" s="51" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="G94" s="51" t="inlineStr">
@@ -6587,17 +6595,17 @@
       </c>
       <c r="H94" s="51" t="inlineStr">
         <is>
-          <t>Plan 22, secciones 3.5 y 3.7; plan 19, 3.5.</t>
+          <t>Hecha la pantalla de embudo (rama feat/panel-interno-metricas).</t>
         </is>
       </c>
       <c r="I94" s="51" t="inlineStr">
         <is>
-          <t>Antes del arranque del piloto.</t>
+          <t>Falta: preguntas del registro (días de apertura, experiencia digital), párrafo de la política de datos (texto legal: lo aprueba Luis) y encuesta de satisfacción.</t>
         </is>
       </c>
       <c r="J94" s="51" t="n"/>
       <c r="K94" s="53" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="L94" s="54">
         <f>IF(K94="","",TODAY()-K94)</f>
@@ -7327,7 +7335,7 @@
       </c>
       <c r="F108" s="51" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>Por verificar</t>
         </is>
       </c>
       <c r="G108" s="51" t="inlineStr">
@@ -7337,17 +7345,17 @@
       </c>
       <c r="H108" s="51" t="inlineStr">
         <is>
-          <t>Plan 22, sección 3.3.</t>
+          <t>Tienda.es_prueba (migración) y botón «Marcar como tienda de prueba» en el detalle de la tienda, con confirmación y rastro en la bitácora. Las vistas de activación y adopción la excluyen.</t>
         </is>
       </c>
       <c r="I108" s="51" t="inlineStr">
         <is>
-          <t>Antes del arranque del piloto, junto con I2.</t>
+          <t>Antes del arranque: marcar en producción las tiendas del equipo (QA, demostración, admin/admin123).</t>
         </is>
       </c>
       <c r="J108" s="51" t="n"/>
       <c r="K108" s="53" t="n">
-        <v>46293</v>
+        <v>46303</v>
       </c>
       <c r="L108" s="54">
         <f>IF(K108="","",TODAY()-K108)</f>
@@ -8554,6 +8562,301 @@
       </c>
       <c r="L129" s="54">
         <f>IF(K129="","",TODAY()-K129)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130" ht="23.85" customHeight="1" s="33">
+      <c r="A130" s="51" t="inlineStr">
+        <is>
+          <t>P22-20</t>
+        </is>
+      </c>
+      <c r="B130" s="52" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C130" s="51" t="inlineStr">
+        <is>
+          <t>Panel interno</t>
+        </is>
+      </c>
+      <c r="D130" s="51" t="inlineStr">
+        <is>
+          <t>Confirmar dos definiciones PROPUESTAS del panel: el umbral «regular» de la adopción (50 %) y qué es «con uso en la semana 4» (≥ 1 día con ventas entre los días 22 y 28)</t>
+        </is>
+      </c>
+      <c r="E130" s="51" t="inlineStr">
+        <is>
+          <t>Decisión pendiente</t>
+        </is>
+      </c>
+      <c r="F130" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G130" s="51" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H130" s="51" t="inlineStr">
+        <is>
+          <t>services/interno/definiciones.js (UMBRAL_ADOPCION_REGULAR, SEMANA_DEL_EMBUDO); plan 22, «I1 e I2 — Resultados».</t>
+        </is>
+      </c>
+      <c r="I130" s="51" t="inlineStr">
+        <is>
+          <t>Fijar ANTES de publicar la convocatoria (documento de intervención, sección 1.6).</t>
+        </is>
+      </c>
+      <c r="J130" s="51" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K130" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L130" s="54">
+        <f>IF(K130="","",TODAY()-K130)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131" ht="23.85" customHeight="1" s="33">
+      <c r="A131" s="51" t="inlineStr">
+        <is>
+          <t>P22-21</t>
+        </is>
+      </c>
+      <c r="B131" s="52" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C131" s="51" t="inlineStr">
+        <is>
+          <t>Panel interno</t>
+        </is>
+      </c>
+      <c r="D131" s="51" t="inlineStr">
+        <is>
+          <t>Confirmar qué cuenta como «productos cargados» en la activación: los que tiene la tienda (hoy) o solo los cargados en sus primeros 7 días</t>
+        </is>
+      </c>
+      <c r="E131" s="51" t="inlineStr">
+        <is>
+          <t>Decisión pendiente</t>
+        </is>
+      </c>
+      <c r="F131" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G131" s="51" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H131" s="51" t="inlineStr">
+        <is>
+          <t>interno.v_activacion expone ambos (productos_cargados y productos_primeros_7d); el cambio es una línea en services/interno/definiciones.js.</t>
+        </is>
+      </c>
+      <c r="I131" s="51" t="inlineStr">
+        <is>
+          <t>La decisión del 28-sep dice «carga al menos 20 productos» sin ventana.</t>
+        </is>
+      </c>
+      <c r="J131" s="51" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K131" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L131" s="54">
+        <f>IF(K131="","",TODAY()-K131)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132" ht="23.85" customHeight="1" s="33">
+      <c r="A132" s="51" t="inlineStr">
+        <is>
+          <t>P22-22</t>
+        </is>
+      </c>
+      <c r="B132" s="52" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C132" s="51" t="inlineStr">
+        <is>
+          <t>Panel interno</t>
+        </is>
+      </c>
+      <c r="D132" s="51" t="inlineStr">
+        <is>
+          <t>Crear las cuentas del equipo en producción y marcar las tiendas de prueba, una vez desplegado el panel</t>
+        </is>
+      </c>
+      <c r="E132" s="51" t="inlineStr">
+        <is>
+          <t>Pendiente del plan</t>
+        </is>
+      </c>
+      <c r="F132" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G132" s="51" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H132" s="51" t="inlineStr">
+        <is>
+          <t>docs/Protocolo_Produccion.md, sección 6 (npm run equipo:crear con la URL de Neon, copia de seguridad antes).</t>
+        </is>
+      </c>
+      <c r="I132" s="51" t="inlineStr">
+        <is>
+          <t>Una cuenta por integrante. Revisar en los logs de Render que la migración terminó bien.</t>
+        </is>
+      </c>
+      <c r="J132" s="51" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K132" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L132" s="54">
+        <f>IF(K132="","",TODAY()-K132)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133" ht="23.85" customHeight="1" s="33">
+      <c r="A133" s="51" t="inlineStr">
+        <is>
+          <t>P22-23</t>
+        </is>
+      </c>
+      <c r="B133" s="52" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C133" s="51" t="inlineStr">
+        <is>
+          <t>Panel interno</t>
+        </is>
+      </c>
+      <c r="D133" s="51" t="inlineStr">
+        <is>
+          <t>Aprobar y publicar el párrafo de la política de datos (plan 22, 3.7) que informa las métricas agregadas y que cada consulta del equipo queda registrada</t>
+        </is>
+      </c>
+      <c r="E133" s="51" t="inlineStr">
+        <is>
+          <t>Decisión pendiente</t>
+        </is>
+      </c>
+      <c r="F133" s="51" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G133" s="51" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H133" s="51" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/PoliticaDatosPage.jsx. Es un texto legal: no se modificó sin el visto bueno de Luis.</t>
+        </is>
+      </c>
+      <c r="I133" s="51" t="inlineStr">
+        <is>
+          <t>Antes de la convocatoria.</t>
+        </is>
+      </c>
+      <c r="J133" s="51" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K133" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L133" s="54">
+        <f>IF(K133="","",TODAY()-K133)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134" ht="23.85" customHeight="1" s="33">
+      <c r="A134" s="51" t="inlineStr">
+        <is>
+          <t>P21-29</t>
+        </is>
+      </c>
+      <c r="B134" s="52" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C134" s="51" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="D134" s="51" t="inlineStr">
+        <is>
+          <t>Carrera latente en las pruebas de integración: helpers/db.js cargaba su propia copia de config/database.js y truncaba mientras esa copia migraba (deadlock intermitente)</t>
+        </is>
+      </c>
+      <c r="E134" s="51" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F134" s="51" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G134" s="51" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H134" s="51" t="inlineStr">
+        <is>
+          <t>Corregido en la rama feat/panel-interno-metricas: el helper espera su migración. 60 corridas seguidas sin fallos.</t>
+        </is>
+      </c>
+      <c r="I134" s="51" t="inlineStr">
+        <is>
+          <t>Falta mezclar a main.</t>
+        </is>
+      </c>
+      <c r="J134" s="51" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K134" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L134" s="54">
+        <f>IF(K134="","",TODAY()-K134)</f>
         <v/>
       </c>
     </row>
@@ -8625,7 +8928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="32" min="1" max="1"/>
@@ -9128,6 +9431,36 @@
       <c r="F19" s="32" t="inlineStr">
         <is>
           <t>Revisión del 2FA del commit ec4d48c: era solo frontend. Luis decide que en el piloto el 2FA se informa pero no se exige, y aprueba mover el control al servidor como política apagada por defecto (REQUIRE_ADMIN_2FA). Rama feat/2fa-politica-servidor (política en el servidor, 409 en generate2FA, limitador, aviso en el frontend). Pendiente: mezclar a main, códigos de recuperación antes de encender la política.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" s="33">
+      <c r="A20" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>P22-02, P22-03, P22-05, P22-19 a P22-23, P21-29</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>Por verificar / Parcial / No iniciado</t>
+        </is>
+      </c>
+      <c r="E20" s="32" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="F20" s="32" t="inlineStr">
+        <is>
+          <t>Luis pide implementar las métricas de la pantalla del superusuario para medir las tiendas del piloto, «o al menos la única que acepte usarla». Implementados I1, I2 y la pantalla de embudo en la rama feat/panel-interno-metricas (esquema interno, cuentas del equipo con 2FA por script, vistas, Tiendas/Detalle/Embudo/Bitácora); funciona con una sola tienda. Pendientes de Luis: 3 definiciones propuestas (P22-20, P22-21), el párrafo legal de la política de datos (P22-23) y crear las cuentas en producción (P22-22). Queda de I4: preguntas del registro y encuesta.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(demo): tienda de demostracion reproducible y siembra con guardia (plan 25, fase 1)
- database/demoEscenario.js: escenario puro (hoy + semilla): 28 productos, 207 ventas, fiado, caja de ayer cerrada,
  tres pedidos (aprobado, borrador, enviado) y Kardex, con las alertas de stock y vencimiento que promete el guion.
- database/seed_demo.js + npm run demo:sembrar: vacia las tablas de la app (no interno.*) y siembra en una transaccion;
  solo corre contra un host local y una base que termine en _demo; exige DEMO_PASSWORD; espera db.migrationReady.
- Pruebas: 23 + 7 unitarias y 19 de integracion; mutaciones comprobadas; recorrido manual en una base local.
- Plan 25 con los resultados y el seguimiento actualizado (P25-04 terminado, P22-27 nuevo).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$4:$L$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$4:$L$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -1759,7 +1759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L155"/>
+  <dimension ref="A1:L156"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="34" min="1" max="1"/>
@@ -8836,7 +8836,7 @@
       </c>
       <c r="I132" s="53" t="inlineStr">
         <is>
-          <t>Una cuenta por integrante. Revisar en los logs de Render que la migración terminó bien.</t>
+          <t>Una cuenta por integrante. Revisar en los logs de Render que la migración terminó bien. Antes de crear las cuentas de producción hay que mezclar fix/equipo-crear-aviso-contrasena (P22-27): con Node 24 el script mostraba la contraseña al teclearla.</t>
         </is>
       </c>
       <c r="J132" s="53" t="inlineStr">
@@ -8845,7 +8845,7 @@
         </is>
       </c>
       <c r="K132" s="55" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="L132" s="56">
         <f>IF(K132="","",TODAY()-K132)</f>
@@ -9934,7 +9934,7 @@
       </c>
       <c r="F151" s="53" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="G151" s="53" t="inlineStr">
@@ -9944,12 +9944,12 @@
       </c>
       <c r="H151" s="53" t="inlineStr">
         <is>
-          <t>Plan 25, fase 1. Hoy la semilla (seed_test_data.js) usa Math.random y no deja alertas de vencimiento, borradores ni proveedor con correo.</t>
+          <t>Hecha el 9-oct-2026 en feat/tienda-demo: database/demoEscenario.js, database/seed_demo.js, npm run demo:sembrar. Pruebas: demo_escenario (23), demo_guardia (7), demo_sembrado (19, integración); suites completas 444 unitarias y 569 de integración en verde; mutaciones detectadas; recorrido manual en el navegador con una base local stockpilot_demo. Resultados en el plan 25, sección 4.</t>
         </is>
       </c>
       <c r="I151" s="53" t="inlineStr">
         <is>
-          <t>Listo para empezar tras el commit de docs (D7). Revisión /review-plan del 9-oct aplicada al plan.</t>
+          <t>No cubierto: quitar await db.migrationReady (intermitente); envío real de correo; celular. Falta el commit/merge a main (con aprobación de Luis).</t>
         </is>
       </c>
       <c r="J151" s="53" t="inlineStr">
@@ -10008,7 +10008,7 @@
       </c>
       <c r="I152" s="53" t="inlineStr">
         <is>
-          <t>Espera P25-04. Responsable Equipo (el ensayo lo hace una persona que no escribió el guion).</t>
+          <t>Listo para empezar: P25-04 hecha. Debe incluir la plantilla de .env.demo (no se pudo crear .env.demo.example: regla de permisos), el ensayo cronometrado y las notas de «Cosas a tener presentes» del plan 25.</t>
         </is>
       </c>
       <c r="J152" s="53" t="inlineStr">
@@ -10201,8 +10201,67 @@
         <v/>
       </c>
     </row>
+    <row r="156" ht="66.75" customHeight="1" s="35">
+      <c r="A156" s="53" t="inlineStr">
+        <is>
+          <t>P22-27</t>
+        </is>
+      </c>
+      <c r="B156" s="54" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C156" s="53" t="inlineStr">
+        <is>
+          <t>Panel interno</t>
+        </is>
+      </c>
+      <c r="D156" s="53" t="inlineStr">
+        <is>
+          <t>npm run equipo:crear: en Node 24 la contraseña se veía al teclearla y el aviso «Contraseña…» se borraba (la pantalla parecía detenida en «Usuario»)</t>
+        </is>
+      </c>
+      <c r="E156" s="53" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F156" s="53" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G156" s="53" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H156" s="53" t="inlineStr">
+        <is>
+          <t>Corregido el 9-oct-2026 en fix/equipo-crear-aviso-contrasena (commit d176576): services/interno/entradaOculta.js + scripts/equipo_crear.js. Prueba: tests/business_logic/entrada_oculta.test.js (readline real en modo terminal; la implementación anterior queda como referencia). Verificado por tubería contra stockpilot_test.</t>
+        </is>
+      </c>
+      <c r="I156" s="53" t="inlineStr">
+        <is>
+          <t>Por verificar en una terminal real de Luis (el defecto se encontró ahí). Aún no está en main; hace falta mezclar la rama antes de crear las cuentas de producción (P22-22).</t>
+        </is>
+      </c>
+      <c r="J156" s="53" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K156" s="55" t="n">
+        <v>46304</v>
+      </c>
+      <c r="L156" s="56">
+        <f>IF(K156="","",TODAY()-K156)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L155"/>
+  <autoFilter ref="A4:L156"/>
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>
@@ -11166,14 +11225,64 @@
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="35">
-      <c r="C33" s="34" t="n"/>
-      <c r="D33" s="34" t="n"/>
-      <c r="E33" s="34" t="n"/>
+      <c r="A33" s="55" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t>P25-04, P25-05</t>
+        </is>
+      </c>
+      <c r="C33" s="34" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="D33" s="34" t="inlineStr">
+        <is>
+          <t>Terminado / No iniciado</t>
+        </is>
+      </c>
+      <c r="E33" s="34" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>Fase 1 del plan 25 hecha en feat/tienda-demo (escenario puro, siembra con guardia _demo, 49 pruebas nuevas entre unitarias e integración, mutaciones y recorrido manual en el navegador). Suites completas: 444 unitarias y 569 de integración en verde. Ajuste: los pedidos de la demo llevan productos distintos de los que /pedir sugiere. Sin push.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="35">
-      <c r="C34" s="34" t="n"/>
-      <c r="D34" s="34" t="n"/>
-      <c r="E34" s="34" t="n"/>
+      <c r="A34" s="55" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B34" s="34" t="inlineStr">
+        <is>
+          <t>P22-27, P22-22</t>
+        </is>
+      </c>
+      <c r="C34" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D34" s="34" t="inlineStr">
+        <is>
+          <t>Por verificar / No iniciado</t>
+        </is>
+      </c>
+      <c r="E34" s="34" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>Luis ejecutó npm run equipo:crear y la pantalla parecía detenida en «Usuario». Causa: en Node 24 rl._writeToOutput no existe, así que el eco no se silenciaba y el aviso de la contraseña se borraba. Corregido en fix/equipo-crear-aviso-contrasena (d176576, sin push) con una prueba de readline real; verificado por tubería, falta confirmarlo en la terminal de Luis. P22-22 espera esa mezcla.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="35">
       <c r="C35" s="34" t="n"/>

</xml_diff>

<commit_message>
docs(demo): guion de la visita y resultados de la fase 2 (plan 25)
- docs/guion_demo_tienda.md: preparacion unica (base local, plantilla de .env.demo), checklist del dia, guion de 10 pasos con los
  rotulos exactos de la pantalla, plan B y lo que no se ensena. Ensayado en el navegador sobre una base temporal.
- Plan 25: resultados de la fase 2 y hallazgos (P25-09: /pedir vuelve a sugerir lo ya aprobado; P25-10: el mensaje opcional al
  proveedor no se envia). Seguimiento actualizado; enlace desde la guia de entorno.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$4:$L$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$4:$L$162</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -1759,7 +1759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L160"/>
+  <dimension ref="A1:L162"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="34" min="1" max="1"/>
@@ -9993,7 +9993,7 @@
       </c>
       <c r="F152" s="53" t="inlineStr">
         <is>
-          <t>No iniciado</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="G152" s="53" t="inlineStr">
@@ -10003,12 +10003,12 @@
       </c>
       <c r="H152" s="53" t="inlineStr">
         <is>
-          <t>Plan 25, fase 2. Entregable de plan 22, sección 5, A.2.</t>
+          <t>Guion hecho el 9-oct-2026: docs/guion_demo_tienda.md (preparación, checklist del día, 10 pasos con rótulos exactos, plan B, lo que no se enseña). npm run demo:servidor. Ensayo técnico en el navegador con una base temporal (aprobar, recibir parcial, enviar sin correo, caja, venta, arqueo, cartera). Plan 25, sección 4, «Fase 2 — Resultados».</t>
         </is>
       </c>
       <c r="I152" s="53" t="inlineStr">
         <is>
-          <t>Listo para empezar: P25-04 hecha. Debe incluir la plantilla de .env.demo (no se pudo crear .env.demo.example: regla de permisos), el ensayo cronometrado y las notas de «Cosas a tener presentes» del plan 25.</t>
+          <t>Falta: ensayo cronometrado por otra persona, correo real al buzón, celular, venta fiada/egreso/historial en pantalla, camino PDF / «ya la envié».</t>
         </is>
       </c>
       <c r="J152" s="53" t="inlineStr">
@@ -10492,8 +10492,126 @@
         <v/>
       </c>
     </row>
+    <row r="161" ht="66.75" customHeight="1" s="35">
+      <c r="A161" s="53" t="inlineStr">
+        <is>
+          <t>P25-09</t>
+        </is>
+      </c>
+      <c r="B161" s="54" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C161" s="53" t="inlineStr">
+        <is>
+          <t>Demostración</t>
+        </is>
+      </c>
+      <c r="D161" s="53" t="inlineStr">
+        <is>
+          <t>En /pedir, tras aprobar un pedido la lista «Por pedir» vuelve a sugerir los mismos productos (el motor solo descuenta lo que está en borrador, no lo aprobado ni lo enviado que aún no llegó)</t>
+        </is>
+      </c>
+      <c r="E161" s="53" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F161" s="53" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G161" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H161" s="53" t="inlineStr">
+        <is>
+          <t>Ensayo del 9-oct-2026 (plan 25, fase 2). Frontend: frontend/src/utils/pedir.js (sugerenciasDePedido recibe el snapshot y el resumen de borradores).</t>
+        </is>
+      </c>
+      <c r="I161" s="53" t="inlineStr">
+        <is>
+          <t>El guion avisa cómo explicarlo. Decidir si las órdenes Aprobadas/Enviadas/Parcial también descuentan (y cuánto, según lo pendiente de recibir).</t>
+        </is>
+      </c>
+      <c r="J161" s="53" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K161" s="55" t="n">
+        <v>46304</v>
+      </c>
+      <c r="L161" s="56">
+        <f>IF(K161="","",TODAY()-K161)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162" ht="66.75" customHeight="1" s="35">
+      <c r="A162" s="53" t="inlineStr">
+        <is>
+          <t>P25-10</t>
+        </is>
+      </c>
+      <c r="B162" s="54" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C162" s="53" t="inlineStr">
+        <is>
+          <t>Demostración</t>
+        </is>
+      </c>
+      <c r="D162" s="53" t="inlineStr">
+        <is>
+          <t>El campo «Mensaje para el proveedor (opcional)» del detalle de la orden no se envía: el frontend manda mensaje_personalizado y el backend nunca lo lee</t>
+        </is>
+      </c>
+      <c r="E162" s="53" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F162" s="53" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G162" s="53" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="H162" s="53" t="inlineStr">
+        <is>
+          <t>frontend/src/hooks/useProveedoresPage.js:255 lo envía; controllers/suppliersController.js (sendOrderToSupplier) no lo usa (búsqueda en controllers, routes, services y models: sin resultados).</t>
+        </is>
+      </c>
+      <c r="I162" s="53" t="inlineStr">
+        <is>
+          <t>Incluirlo en el correo o quitar el campo. Relacionado con P25-06 (mismo endpoint).</t>
+        </is>
+      </c>
+      <c r="J162" s="53" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K162" s="55" t="n">
+        <v>46304</v>
+      </c>
+      <c r="L162" s="56">
+        <f>IF(K162="","",TODAY()-K162)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L160"/>
+  <autoFilter ref="A4:L162"/>
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>
@@ -11577,9 +11695,34 @@
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="35">
-      <c r="C37" s="34" t="n"/>
-      <c r="D37" s="34" t="n"/>
-      <c r="E37" s="34" t="n"/>
+      <c r="A37" s="55" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B37" s="34" t="inlineStr">
+        <is>
+          <t>P25-05, P25-09, P25-10</t>
+        </is>
+      </c>
+      <c r="C37" s="34" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="D37" s="34" t="inlineStr">
+        <is>
+          <t>Parcial / No iniciado</t>
+        </is>
+      </c>
+      <c r="E37" s="34" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>Fase 2 del plan 25: guion de la visita (docs/guion_demo_tienda.md) y ensayo técnico en el navegador sobre una base temporal. Hallazgos: «Por pedir» vuelve a sugerir lo ya aprobado (P25-09) y el mensaje opcional al proveedor no se envía (P25-10). Falta el ensayo cronometrado por otra persona, el correo real y el celular.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="35">
       <c r="C38" s="34" t="n"/>

</xml_diff>

<commit_message>
docs(seguimiento): filas del plan 26, alertas al ingresar y tras carga masiva, recalculo por tiempo y bitacora
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento_planes.xlsx
+++ b/docs/seguimiento_planes.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$4:$L$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$4:$L$170</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -898,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="34" min="1" max="1"/>
@@ -1737,6 +1737,34 @@
       </c>
       <c r="J27" s="40">
         <f>COUNTIF(Pendientes!$B$5:$B$308,E27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" s="42" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="F28" s="40" t="inlineStr">
+        <is>
+          <t>Dispositivos de confianza para el 2FA</t>
+        </is>
+      </c>
+      <c r="G28" s="40">
+        <f>COUNTIFS(Pendientes!$B$5:$B$308,E28,Pendientes!$F$5:$F$308,"&lt;&gt;Terminado",Pendientes!$F$5:$F$308,"&lt;&gt;Descartado")-COUNTIFS(Pendientes!$B$5:$B$308,E28,Pendientes!$F$5:$F$308,"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="40">
+        <f>COUNTIFS(Pendientes!$B$5:$B$308,E28,Pendientes!$F$5:$F$308,"Terminado")</f>
+        <v/>
+      </c>
+      <c r="I28" s="40">
+        <f>COUNTIFS(Pendientes!$B$5:$B$308,E28,Pendientes!$F$5:$F$308,"Descartado")</f>
+        <v/>
+      </c>
+      <c r="J28" s="40">
+        <f>COUNTIF(Pendientes!$B$5:$B$308,E28)</f>
         <v/>
       </c>
     </row>
@@ -1759,7 +1787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L163"/>
+  <dimension ref="A1:L170"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="34" min="1" max="1"/>
@@ -1779,14 +1807,14 @@
     <row r="1" ht="17.25" customHeight="1" s="35">
       <c r="A1" s="36" t="inlineStr">
         <is>
-          <t>StockPilot · Seguimiento de pendientes de los planes 02 a 25</t>
+          <t>StockPilot · Seguimiento de pendientes de los planes 02 a 26</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="35">
       <c r="A2" s="37" t="inlineStr">
         <is>
-          <t>Revisado contra el código y el historial de git (main y origin/main) el 09-10-2026. Cambie el Estado con la lista desplegable y anote la fecha, quién y qué en la Bitácora. Los planes 01 y 03 no tienen pendientes.</t>
+          <t>Revisado contra el código y el historial de git (main y origin/main) el 10-10-2026. Cambie el Estado con la lista desplegable y anote la fecha, quién y qué en la Bitácora. Los planes 01 y 03 no tienen pendientes.</t>
         </is>
       </c>
     </row>
@@ -10669,8 +10697,421 @@
         <v/>
       </c>
     </row>
+    <row r="164" ht="66.75" customHeight="1" s="35">
+      <c r="A164" s="53" t="inlineStr">
+        <is>
+          <t>P17-08</t>
+        </is>
+      </c>
+      <c r="B164" s="54" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C164" s="53" t="inlineStr">
+        <is>
+          <t>Alertas</t>
+        </is>
+      </c>
+      <c r="D164" s="53" t="inlineStr">
+        <is>
+          <t>Las alertas de la tienda quedaban desactualizadas hasta que alguien abría el Monitor: al ingresar a la app no se recalculaban</t>
+        </is>
+      </c>
+      <c r="E164" s="53" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F164" s="53" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G164" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H164" s="53" t="inlineStr">
+        <is>
+          <t>Corregido el 10-oct-2026 en fix/alertas-al-ingresar (commit f6b4069), mezclado a main (dd26501, c346f80) y subido: services/alertas/refrescoAlEntrar.js, llamado desde authController.js en el login y en verify2FA. Espera como máximo 3 s y nunca rompe el inicio de sesión. Pruebas: tests/business_logic/refresco_alertas_al_entrar.test.js y tests/integration/login_refresca_alertas.test.js. Unitarias 476 en verde; integración completa sobre la rama: 53 archivos y 584 pruebas en verde (corrida de Luis).</t>
+        </is>
+      </c>
+      <c r="I164" s="53" t="inlineStr">
+        <is>
+          <t>Por verificar por Luis en producción tras el despliegue de Render (ingresar y ver la campanita y el Monitor al día). No cambia la API ni el contrato [A1].</t>
+        </is>
+      </c>
+      <c r="J164" s="53" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K164" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="L164" s="56">
+        <f>IF(K164="","",TODAY()-K164)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165" ht="66.75" customHeight="1" s="35">
+      <c r="A165" s="53" t="inlineStr">
+        <is>
+          <t>P17-09</t>
+        </is>
+      </c>
+      <c r="B165" s="54" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C165" s="53" t="inlineStr">
+        <is>
+          <t>Alertas</t>
+        </is>
+      </c>
+      <c r="D165" s="53" t="inlineStr">
+        <is>
+          <t>La carga masiva de productos no recalculaba las alertas de la tienda</t>
+        </is>
+      </c>
+      <c r="E165" s="53" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F165" s="53" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G165" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H165" s="53" t="inlineStr">
+        <is>
+          <t>Corregido el 10-oct-2026 en fix/alertas-al-ingresar (commit 554c8b2): controllers/productController.js recalcula las alertas al terminar la carga. Prueba: tests/integration/carga_masiva_alertas.test.js (dentro de las 584 de la integración completa en verde). Mezclado a main (dd26501, c346f80).</t>
+        </is>
+      </c>
+      <c r="I165" s="53" t="inlineStr">
+        <is>
+          <t>Por verificar por Luis con una carga masiva real en la tienda de demostración o en producción.</t>
+        </is>
+      </c>
+      <c r="J165" s="53" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K165" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="L165" s="56">
+        <f>IF(K165="","",TODAY()-K165)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166" ht="66.75" customHeight="1" s="35">
+      <c r="A166" s="53" t="inlineStr">
+        <is>
+          <t>P17-10</t>
+        </is>
+      </c>
+      <c r="B166" s="54" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C166" s="53" t="inlineStr">
+        <is>
+          <t>Alertas</t>
+        </is>
+      </c>
+      <c r="D166" s="53" t="inlineStr">
+        <is>
+          <t>Las alertas por vencimiento no se recalculan por el solo paso del tiempo: no hay tarea periódica, solo se refrescan al ocurrir un evento (ingreso a la app, carga masiva, etc.)</t>
+        </is>
+      </c>
+      <c r="E166" s="53" t="inlineStr">
+        <is>
+          <t>Observación / defecto</t>
+        </is>
+      </c>
+      <c r="F166" s="53" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G166" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H166" s="53" t="inlineStr">
+        <is>
+          <t>Detectado el 10-oct-2026 al corregir P17-08 y P17-09. Hoy el recálculo depende de que alguien ingrese o cargue productos; un lote que pasa a «por vencer» solo porque pasan los días no genera alerta hasta el siguiente refresco. A confirmar contra el código antes de implementar.</t>
+        </is>
+      </c>
+      <c r="I166" s="53" t="inlineStr">
+        <is>
+          <t>Decidir si se resuelve con una tarea periódica (cron o planificador del hospedaje) o con el refresco al ingresar que ya existe. Una tarea periódica añade infraestructura y puede tocar producción: decide Luis.</t>
+        </is>
+      </c>
+      <c r="J166" s="53" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K166" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="L166" s="56">
+        <f>IF(K166="","",TODAY()-K166)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="167" ht="66.75" customHeight="1" s="35">
+      <c r="A167" s="53" t="inlineStr">
+        <is>
+          <t>P26-01</t>
+        </is>
+      </c>
+      <c r="B167" s="54" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C167" s="53" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D167" s="53" t="inlineStr">
+        <is>
+          <t>Plan 26 (dispositivos de confianza para el 2FA): decisiones D1 a D7 (roles, canal de la app, número de dispositivos, aviso por correo, señal del navegador, qué hace cerrar sesión, fecha)</t>
+        </is>
+      </c>
+      <c r="E167" s="53" t="inlineStr">
+        <is>
+          <t>Decisión pendiente</t>
+        </is>
+      </c>
+      <c r="F167" s="53" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G167" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H167" s="53" t="inlineStr">
+        <is>
+          <t>docs/planes/26_dispositivos_de_confianza_2fa.md (propuesta sin implementar, mezclada a main el 10-oct-2026, c346f80). Ya decididas por Luis: máximo 15 días, pedir 2FA desde otro dispositivo, priorizar las vulnerabilidades.</t>
+        </is>
+      </c>
+      <c r="I167" s="53" t="inlineStr">
+        <is>
+          <t>Recomendación del plan: D7 = después del piloto, junto con los códigos de recuperación (P21-26) y REQUIRE_ADMIN_2FA. Toca autenticación y esquema: alto riesgo, no se empieza sin aprobación.</t>
+        </is>
+      </c>
+      <c r="J167" s="53" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
+      <c r="K167" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="L167" s="56">
+        <f>IF(K167="","",TODAY()-K167)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168" ht="66.75" customHeight="1" s="35">
+      <c r="A168" s="53" t="inlineStr">
+        <is>
+          <t>P26-02</t>
+        </is>
+      </c>
+      <c r="B168" s="54" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C168" s="53" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D168" s="53" t="inlineStr">
+        <is>
+          <t>Plan 26, fase 1: tabla dispositivos_confianza (hash del token, rotación, detección de reutilización) y reglas puras con pruebas, sin tocar el login</t>
+        </is>
+      </c>
+      <c r="E168" s="53" t="inlineStr">
+        <is>
+          <t>Trabajo futuro</t>
+        </is>
+      </c>
+      <c r="F168" s="53" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G168" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H168" s="53" t="inlineStr">
+        <is>
+          <t>docs/planes/26_dispositivos_de_confianza_2fa.md, sección 5. Migración aditiva e idempotente (skill safe-migrations); archivos nuevos config/migraciones/dispositivosConfianza.js y services/seguridad/dispositivosConfianza.js.</t>
+        </is>
+      </c>
+      <c r="I168" s="53" t="inlineStr">
+        <is>
+          <t>Depende de P26-01. Pruebas primero y mutación de cada defensa (token en claro, sin rotar, sin validar el usuario).</t>
+        </is>
+      </c>
+      <c r="J168" s="53" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K168" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="L168" s="56">
+        <f>IF(K168="","",TODAY()-K168)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169" ht="66.75" customHeight="1" s="35">
+      <c r="A169" s="53" t="inlineStr">
+        <is>
+          <t>P26-03</t>
+        </is>
+      </c>
+      <c r="B169" s="54" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C169" s="53" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D169" s="53" t="inlineStr">
+        <is>
+          <t>Plan 26, fase 2: integrar con login y verify2FA; la cookie nunca sustituye la contraseña</t>
+        </is>
+      </c>
+      <c r="E169" s="53" t="inlineStr">
+        <is>
+          <t>Trabajo futuro</t>
+        </is>
+      </c>
+      <c r="F169" s="53" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G169" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H169" s="53" t="inlineStr">
+        <is>
+          <t>docs/planes/26_dispositivos_de_confianza_2fa.md, sección 5. Cookie HttpOnly, SameSite=Strict, Secure en producción, máximo 15 días. Prueba obligatoria: cookie válida con contraseña mala = 401 sin sesión, y authLimiter sigue contando.</t>
+        </is>
+      </c>
+      <c r="I169" s="53" t="inlineStr">
+        <is>
+          <t>Depende de P26-02. Parar y preguntar si hay que cambiar el contrato de la app o el orden de findByCredentials.</t>
+        </is>
+      </c>
+      <c r="J169" s="53" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K169" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="L169" s="56">
+        <f>IF(K169="","",TODAY()-K169)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170" ht="66.75" customHeight="1" s="35">
+      <c r="A170" s="53" t="inlineStr">
+        <is>
+          <t>P26-04</t>
+        </is>
+      </c>
+      <c r="B170" s="54" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C170" s="53" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D170" s="53" t="inlineStr">
+        <is>
+          <t>Plan 26, fase 3: revocación (cambio de contraseña, desactivar 2FA), lista en «Mi perfil», aviso por correo, política de datos y /security-review</t>
+        </is>
+      </c>
+      <c r="E170" s="53" t="inlineStr">
+        <is>
+          <t>Trabajo futuro</t>
+        </is>
+      </c>
+      <c r="F170" s="53" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="G170" s="53" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="H170" s="53" t="inlineStr">
+        <is>
+          <t>docs/planes/26_dispositivos_de_confianza_2fa.md, secciones 3 y 5. Revocar en las tres rutas que llaman a User.updatePassword y en disable2FA; actualizar la política de datos (Ley 1581) y el Protocolo.</t>
+        </is>
+      </c>
+      <c r="I170" s="53" t="inlineStr">
+        <is>
+          <t>Depende de P26-03. Salida: /security-review sin hallazgos altos abiertos.</t>
+        </is>
+      </c>
+      <c r="J170" s="53" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="K170" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="L170" s="56">
+        <f>IF(K170="","",TODAY()-K170)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L163"/>
+  <autoFilter ref="A4:L170"/>
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>
@@ -11814,19 +12255,94 @@
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="35">
-      <c r="C39" s="34" t="n"/>
-      <c r="D39" s="34" t="n"/>
-      <c r="E39" s="34" t="n"/>
+      <c r="A39" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B39" s="34" t="inlineStr">
+        <is>
+          <t>P17-08, P17-09</t>
+        </is>
+      </c>
+      <c r="C39" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D39" s="34" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="E39" s="34" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="F39" s="34" t="inlineStr">
+        <is>
+          <t>Luis pide que las alertas se recalculen al ingresar y tras la carga masiva. Rama fix/alertas-al-ingresar (commits f6b4069 y 554c8b2). Integración completa de Luis: 53 archivos y 584 pruebas en verde. Mezclada con las ramas fix/vista-movil-demo y docs/plan-26-dispositivos-de-confianza a main (--no-ff, c346f80) y subida el 10-oct-2026. Pendiente: verificar el despliegue de Render y en pantalla.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="35">
-      <c r="C40" s="34" t="n"/>
-      <c r="D40" s="34" t="n"/>
-      <c r="E40" s="34" t="n"/>
+      <c r="A40" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B40" s="34" t="inlineStr">
+        <is>
+          <t>P17-10</t>
+        </is>
+      </c>
+      <c r="C40" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D40" s="34" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="E40" s="34" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="F40" s="34" t="inlineStr">
+        <is>
+          <t>Se anota el recálculo por paso del tiempo de los vencimientos (sin tarea periódica), detectado al corregir P17-08. A decidir por Luis.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="35">
-      <c r="C41" s="34" t="n"/>
-      <c r="D41" s="34" t="n"/>
-      <c r="E41" s="34" t="n"/>
+      <c r="A41" s="55" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B41" s="34" t="inlineStr">
+        <is>
+          <t>P26-01, P26-02, P26-03, P26-04</t>
+        </is>
+      </c>
+      <c r="C41" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D41" s="34" t="inlineStr">
+        <is>
+          <t>No iniciado</t>
+        </is>
+      </c>
+      <c r="E41" s="34" t="inlineStr">
+        <is>
+          <t>Agente (Claude Code)</t>
+        </is>
+      </c>
+      <c r="F41" s="34" t="inlineStr">
+        <is>
+          <t>Plan 26 (dispositivos de confianza para el 2FA): propuesta mezclada a main sin implementar (c346f80). Se agregan sus decisiones y tres fases al seguimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="35">
       <c r="C42" s="34" t="n"/>

</xml_diff>